<commit_message>
Drop id columns from Admissions/Progress import
Template and importer resolve students by name+kutir and schools by
name only — no student_id or school_id on 19_Admissions / 20_Progress.
</commit_message>
<xml_diff>
--- a/GRS_Import_Template.xlsx
+++ b/GRS_Import_Template.xlsx
@@ -298,7 +298,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Resolve student by student_id OR (first_name+last_name+kutir_name). school_start_year = integer start year (e.g. 2025), not '2025-26'. admission_class: 5 or 8. Pipeline flags: eligible→form_received→applied→admit_card→appeared→selected→admitted. score_&lt;subject&gt; columns optional (subject name with spaces as underscores).</t>
+        <t>Resolve student by first_name+last_name+kutir_name (no student_id). school_start_year = integer start year. admission_class: 5 or 8. Optional score_&lt;subject&gt; columns.</t>
       </text>
     </comment>
   </commentList>
@@ -313,7 +313,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>academic_year = integer start year. status: enrolled|transferred|dropped_out|graduated.</t>
+        <t>Resolve student by first_name+last_name+kutir_name; school by school_name (no student_id / school_id). academic_year = integer. status: enrolled|transferred|dropped_out|graduated.</t>
       </text>
     </comment>
   </commentList>
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -758,6 +758,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -767,6 +768,7 @@
     </row>
     <row r="4"/>
     <row r="5"/>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -1050,6 +1052,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
@@ -1059,6 +1062,12 @@
     </row>
     <row r="33"/>
     <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A32:F34"/>
@@ -2066,208 +2075,206 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="21" customWidth="1" min="23" max="23"/>
-    <col width="17" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-    <col width="19" customWidth="1" min="27" max="27"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>student_id</t>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>first_name</t>
         </is>
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>first_name</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
           <t>last_name</t>
         </is>
       </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>kutir_name</t>
+        </is>
+      </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>kutir_name</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
           <t>school_name</t>
         </is>
       </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>school_type</t>
+        </is>
+      </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>school_type</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
           <t>school_start_year</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>exam_category_name</t>
+        </is>
+      </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>exam_category_name</t>
+          <t>eligible</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>eligible</t>
+          <t>form_received</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
-          <t>form_received</t>
+          <t>applied</t>
         </is>
       </c>
       <c r="K1" s="6" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>admit_card</t>
         </is>
       </c>
       <c r="L1" s="6" t="inlineStr">
         <is>
-          <t>admit_card</t>
+          <t>appeared</t>
         </is>
       </c>
       <c r="M1" s="6" t="inlineStr">
         <is>
-          <t>appeared</t>
+          <t>no_exam_reason</t>
         </is>
       </c>
       <c r="N1" s="6" t="inlineStr">
         <is>
-          <t>no_exam_reason</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="O1" s="6" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>admitted</t>
         </is>
       </c>
       <c r="P1" s="6" t="inlineStr">
         <is>
-          <t>admitted</t>
+          <t>no_admit_reason</t>
         </is>
       </c>
       <c r="Q1" s="6" t="inlineStr">
         <is>
-          <t>no_admit_reason</t>
+          <t>application_number</t>
         </is>
       </c>
       <c r="R1" s="6" t="inlineStr">
         <is>
-          <t>application_number</t>
+          <t>roll_number</t>
         </is>
       </c>
       <c r="S1" s="6" t="inlineStr">
         <is>
-          <t>roll_number</t>
+          <t>exam_center_name</t>
         </is>
       </c>
       <c r="T1" s="6" t="inlineStr">
         <is>
-          <t>exam_center_name</t>
+          <t>admitted_school_name</t>
         </is>
       </c>
       <c r="U1" s="6" t="inlineStr">
         <is>
-          <t>admitted_school_name</t>
+          <t>admission_class</t>
         </is>
       </c>
       <c r="V1" s="6" t="inlineStr">
         <is>
-          <t>admission_class</t>
+          <t>score_mathematics</t>
         </is>
       </c>
       <c r="W1" s="6" t="inlineStr">
         <is>
-          <t>score_mathematics</t>
+          <t>score_english</t>
         </is>
       </c>
       <c r="X1" s="6" t="inlineStr">
         <is>
-          <t>score_english</t>
+          <t>score_evs</t>
         </is>
       </c>
       <c r="Y1" s="6" t="inlineStr">
         <is>
-          <t>score_evs</t>
+          <t>score_hindi</t>
         </is>
       </c>
       <c r="Z1" s="6" t="inlineStr">
         <is>
-          <t>score_hindi</t>
-        </is>
-      </c>
-      <c r="AA1" s="6" t="inlineStr">
-        <is>
           <t>score_reasoning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n"/>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Ravi</t>
+        </is>
+      </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Ravi</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Kutir No 1</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Kutir No 1</t>
+          <t>Govt HS Raipur</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Govt HS Raipur</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
           <t>EMRS</t>
         </is>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="F2" s="7" t="n">
         <v>2025</v>
       </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Navodaya Class V</t>
+        </is>
+      </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Navodaya Class V</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -2290,59 +2297,54 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N2" s="7" t="n"/>
       <c r="O2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="P2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="Q2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>APP/2025/001</t>
+        </is>
+      </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>APP/2025/001</t>
+          <t>ROLL/2025/001</t>
         </is>
       </c>
       <c r="S2" s="7" t="inlineStr">
         <is>
-          <t>ROLL/2025/001</t>
+          <t>Govt School Center</t>
         </is>
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>Govt School Center</t>
-        </is>
-      </c>
-      <c r="U2" s="7" t="inlineStr">
-        <is>
           <t>EMRS Raipur</t>
         </is>
       </c>
+      <c r="U2" s="7" t="n">
+        <v>5</v>
+      </c>
       <c r="V2" s="7" t="n">
-        <v>5</v>
+        <v>85.5</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>85.5</v>
+        <v>72</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>72</v>
+        <v>68.5</v>
       </c>
       <c r="Y2" s="7" t="n">
-        <v>68.5</v>
+        <v>80</v>
       </c>
       <c r="Z2" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="AA2" s="7" t="n">
         <v>91</v>
       </c>
     </row>
@@ -2358,131 +2360,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>student_id</t>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>first_name</t>
         </is>
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>first_name</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
           <t>last_name</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>kutir_name</t>
         </is>
       </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>school_name</t>
+          <t>academic_year</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>school_id</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>academic_year</t>
+          <t>class_in_year</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>class_in_year</t>
+          <t>transfer_school</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>exit_reason</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
-          <t>transfer_school</t>
+          <t>previous_year_percentage</t>
         </is>
       </c>
       <c r="K1" s="6" t="inlineStr">
         <is>
-          <t>exit_reason</t>
-        </is>
-      </c>
-      <c r="L1" s="6" t="inlineStr">
-        <is>
-          <t>previous_year_percentage</t>
-        </is>
-      </c>
-      <c r="M1" s="6" t="inlineStr">
-        <is>
           <t>remarks</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n"/>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Ravi</t>
+        </is>
+      </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Ravi</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Kutir No 1</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Kutir No 1</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
           <t>EMRS Raipur</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n"/>
-      <c r="G2" s="7" t="n">
+      <c r="E2" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="F2" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>enrolled</t>
         </is>
       </c>
-      <c r="J2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n">
+        <v>78.5</v>
+      </c>
       <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="M2" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Resolve import kutir/cluster lookups hierarchically
Cluster and kutir names are parent-scoped (district / cluster), not
globally unique. Import helpers and sheets that looked up by name alone
now require district_name + cluster_name (optional area_name).
</commit_message>
<xml_diff>
--- a/GRS_Import_Template.xlsx
+++ b/GRS_Import_Template.xlsx
@@ -326,7 +326,7 @@
     <author>KutirGRS</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>visited_by = users.username. physical_vs_registered: Matched|Not Matched. workbook_completion: Upto Date|Partial Upto Date|Not Uptodate. book_availability: Sufficient|Lacking|More than required. Ratings 1–5.</t>
       </text>
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1056,18 +1056,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Notes: school_start_year / academic_year are integers (e.g. 2025), not display ranges like 2025-26. parivaar_presence on Districts defaults to yes. SysAdmin is a valid user title. This _Instructions sheet is ignored by the importer.</t>
+          <t>Notes: school_start_year / academic_year are integers (e.g. 2025), not display ranges like 2025-26. parivaar_presence on Districts defaults to yes. SysAdmin is a valid user title. This _Instructions sheet is ignored by the importer. Cluster names are unique within a district (not globally); kutir names are unique within a cluster. Sheets that look up kutir/cluster require district_name + cluster_name (optional area_name) alongside kutir_name / area_name.</t>
         </is>
       </c>
     </row>
     <row r="33"/>
     <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A32:F34"/>
@@ -1460,7 +1454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1479,7 +1473,12 @@
           <t>area_name</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>district_name</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>userid</t>
         </is>
@@ -1496,7 +1495,12 @@
           <t>North Area</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>asha.mehta</t>
         </is>
@@ -1599,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1636,37 +1640,42 @@
           <t>district_name</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>street</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>pincode</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>donor_name</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>enrollment_5th</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>enrollment_8th</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>userid</t>
         </is>
@@ -1693,33 +1702,38 @@
           <t>Raipur</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>North Area</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>123 Main St</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Chhattisgarh</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>492001</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Rotary Club</t>
         </is>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="J2" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="J2" s="7" t="n">
+      <c r="K2" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>asha.mehta</t>
         </is>
@@ -1846,7 +1860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1882,92 +1896,107 @@
           <t>last_name</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>district_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cluster_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>kutir_name</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>dob</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>category_name</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>sub_category_name</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>father_name</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>mother_name</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>street</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>pincode</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>alt_contact_name</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>alt_contact_phone</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>aadhaar</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>category_cert</t>
         </is>
       </c>
-      <c r="R1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>birth_cert</t>
         </is>
       </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>residence_proof</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>medical</t>
         </is>
@@ -1984,80 +2013,95 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cluster 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>North Area</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Kutir No 1</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>2012-06-15</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>ST</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>ST-A</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>Suresh Sharma</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>Sunita Sharma</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>9876543210</t>
         </is>
       </c>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>Village Rampur</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>492001</t>
         </is>
       </c>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="7" t="inlineStr">
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="T2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="U2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="V2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="W2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2075,7 +2119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2117,122 +2161,137 @@
           <t>last_name</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>district_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cluster_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>kutir_name</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>school_name</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>school_type</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>school_start_year</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>exam_category_name</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>eligible</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>form_received</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>applied</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>admit_card</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>appeared</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>no_exam_reason</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>selected</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>admitted</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>no_admit_reason</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>application_number</t>
         </is>
       </c>
-      <c r="R1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>roll_number</t>
         </is>
       </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>exam_center_name</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>admitted_school_name</t>
         </is>
       </c>
-      <c r="U1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>admission_class</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>score_mathematics</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="Z1" s="6" t="inlineStr">
         <is>
           <t>score_english</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="AA1" s="6" t="inlineStr">
         <is>
           <t>score_evs</t>
         </is>
       </c>
-      <c r="Y1" s="6" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>score_hindi</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="AC1" s="6" t="inlineStr">
         <is>
           <t>score_reasoning</t>
         </is>
@@ -2249,55 +2308,59 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cluster 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>North Area</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Kutir No 1</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Govt HS Raipur</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>EMRS</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="I2" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Navodaya Class V</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="M2" s="7" t="n"/>
       <c r="N2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2311,40 +2374,51 @@
       <c r="P2" s="7" t="n"/>
       <c r="Q2" s="7" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
           <t>APP/2025/001</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="U2" s="7" t="inlineStr">
         <is>
           <t>ROLL/2025/001</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="V2" s="7" t="inlineStr">
         <is>
           <t>Govt School Center</t>
         </is>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="W2" s="7" t="inlineStr">
         <is>
           <t>EMRS Raipur</t>
         </is>
       </c>
-      <c r="U2" s="7" t="n">
+      <c r="X2" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="V2" s="7" t="n">
+      <c r="Y2" s="7" t="n">
         <v>85.5</v>
       </c>
-      <c r="W2" s="7" t="n">
+      <c r="Z2" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="X2" s="7" t="n">
+      <c r="AA2" s="7" t="n">
         <v>68.5</v>
       </c>
-      <c r="Y2" s="7" t="n">
+      <c r="AB2" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="Z2" s="7" t="n">
+      <c r="AC2" s="7" t="n">
         <v>91</v>
       </c>
     </row>
@@ -2360,7 +2434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2387,47 +2461,62 @@
           <t>last_name</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>district_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cluster_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>kutir_name</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>school_name</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>academic_year</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>class_in_year</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>transfer_school</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>exit_reason</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>previous_year_percentage</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
@@ -2444,33 +2533,48 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cluster 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>North Area</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Kutir No 1</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>EMRS Raipur</t>
         </is>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="H2" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="I2" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>enrolled</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="n">
+      <c r="K2" s="7" t="n"/>
+      <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="n">
         <v>78.5</v>
       </c>
-      <c r="K2" s="7" t="n"/>
+      <c r="N2" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2484,7 +2588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2535,328 +2639,349 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>district_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>cluster_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>kutir_name</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>visit_date</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>visited_by</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>avg_attendance_morning</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>avg_attendance_evening</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>follow_timetable</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>kutir_closed</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>plan_hindi</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>plan_math</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>plan_english</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>timetable_plan_reason</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>math_topics_pre</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>math_topics_upper</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>english_topics_pre</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>english_topics_upper</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>timeslot_reason</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>grs_prep_remarks</t>
         </is>
       </c>
-      <c r="R1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>physical_vs_registered</t>
         </is>
       </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>workbook_percentage</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>workbook_completion</t>
         </is>
       </c>
-      <c r="U1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>book_availability</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>cleanliness</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="Z1" s="6" t="inlineStr">
         <is>
           <t>hindi_proficiency</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="AA1" s="6" t="inlineStr">
         <is>
           <t>english_proficiency</t>
         </is>
       </c>
-      <c r="Y1" s="6" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>maths_proficiency</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="AC1" s="6" t="inlineStr">
         <is>
           <t>evs_proficiency</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>reasoning_proficiency</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AE1" s="6" t="inlineStr">
         <is>
           <t>material_management</t>
         </is>
       </c>
-      <c r="AC1" s="6" t="inlineStr">
+      <c r="AF1" s="6" t="inlineStr">
         <is>
           <t>kutir_performance</t>
         </is>
       </c>
-      <c r="AD1" s="6" t="inlineStr">
+      <c r="AG1" s="6" t="inlineStr">
         <is>
           <t>staff_behavior</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>reg_admission_forms</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AI1" s="6" t="inlineStr">
         <is>
           <t>reg_attendance_students</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AJ1" s="6" t="inlineStr">
         <is>
           <t>reg_daily_activity</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AK1" s="6" t="inlineStr">
         <is>
           <t>reg_observation</t>
         </is>
       </c>
-      <c r="AI1" s="6" t="inlineStr">
+      <c r="AL1" s="6" t="inlineStr">
         <is>
           <t>reg_students_data</t>
         </is>
       </c>
-      <c r="AJ1" s="6" t="inlineStr">
+      <c r="AM1" s="6" t="inlineStr">
         <is>
           <t>reg_attendance_teachers</t>
         </is>
       </c>
-      <c r="AK1" s="6" t="inlineStr">
+      <c r="AN1" s="6" t="inlineStr">
         <is>
           <t>reg_students_documents</t>
         </is>
       </c>
-      <c r="AL1" s="6" t="inlineStr">
+      <c r="AO1" s="6" t="inlineStr">
         <is>
           <t>regular_students_morning</t>
         </is>
       </c>
-      <c r="AM1" s="6" t="inlineStr">
+      <c r="AP1" s="6" t="inlineStr">
         <is>
           <t>regular_students_evening</t>
         </is>
       </c>
-      <c r="AN1" s="6" t="inlineStr">
+      <c r="AQ1" s="6" t="inlineStr">
         <is>
           <t>timeslot_bal_sabha</t>
         </is>
       </c>
-      <c r="AO1" s="6" t="inlineStr">
+      <c r="AR1" s="6" t="inlineStr">
         <is>
           <t>timeslot_sports</t>
         </is>
       </c>
-      <c r="AP1" s="6" t="inlineStr">
+      <c r="AS1" s="6" t="inlineStr">
         <is>
           <t>timeslot_yoga</t>
         </is>
       </c>
-      <c r="AQ1" s="6" t="inlineStr">
+      <c r="AT1" s="6" t="inlineStr">
         <is>
           <t>timeslot_value_ed</t>
         </is>
       </c>
-      <c r="AR1" s="6" t="inlineStr">
+      <c r="AU1" s="6" t="inlineStr">
         <is>
           <t>timeslot_gk_map</t>
         </is>
       </c>
-      <c r="AS1" s="6" t="inlineStr">
+      <c r="AV1" s="6" t="inlineStr">
         <is>
           <t>final_remarks</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cluster 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>North Area</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Kutir No 1</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>2025-06-15</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>asha.mehta</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="G2" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="H2" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>Addition, Subtraction</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>Fractions, Algebra</t>
         </is>
       </c>
-      <c r="N2" s="7" t="inlineStr">
+      <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>Vowels, Basic words</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>Grammar, Comprehension</t>
         </is>
       </c>
-      <c r="P2" s="7" t="n"/>
-      <c r="Q2" s="7" t="n"/>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>
       </c>
-      <c r="S2" s="7" t="n">
+      <c r="V2" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="W2" s="7" t="inlineStr">
         <is>
           <t>Upto Date</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="X2" s="7" t="inlineStr">
         <is>
           <t>Sufficient</t>
         </is>
-      </c>
-      <c r="V2" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="W2" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="X2" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>4</v>
@@ -2871,76 +2996,85 @@
         <v>4</v>
       </c>
       <c r="AC2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE2" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="AD2" s="7" t="n"/>
-      <c r="AE2" s="7" t="inlineStr">
+      <c r="AF2" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG2" s="7" t="n"/>
+      <c r="AH2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AF2" s="7" t="inlineStr">
+      <c r="AI2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AG2" s="7" t="inlineStr">
+      <c r="AJ2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AH2" s="7" t="inlineStr">
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AI2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AJ2" s="7" t="inlineStr">
+      <c r="AM2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AN2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AL2" s="7" t="n">
+      <c r="AO2" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="AM2" s="7" t="n">
+      <c r="AP2" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="AN2" s="7" t="inlineStr">
+      <c r="AQ2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AO2" s="7" t="inlineStr">
+      <c r="AR2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AP2" s="7" t="inlineStr">
+      <c r="AS2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AQ2" s="7" t="inlineStr">
+      <c r="AT2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AR2" s="7" t="inlineStr">
+      <c r="AU2" s="7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AS2" s="7" t="n"/>
+      <c r="AV2" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Users list pagination and split donor email/phone
Users list uses server-side pagination with batch geo attach.
Donors replace generic contact with email + phone (migration 024,
Lookups UI, field registry, import template).
</commit_message>
<xml_diff>
--- a/GRS_Import_Template.xlsx
+++ b/GRS_Import_Template.xlsx
@@ -758,7 +758,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -768,7 +767,6 @@
     </row>
     <row r="4"/>
     <row r="5"/>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -1052,7 +1050,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
@@ -3206,7 +3203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3222,10 +3219,15 @@
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>email</t>
         </is>
       </c>
       <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -3239,10 +3241,15 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Mr. Gupta / 9876543210</t>
+          <t>sponsor@rotary.example</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Annual sponsor</t>
         </is>

</xml_diff>